<commit_message>
Complete portfolio source audit and cleanup
</commit_message>
<xml_diff>
--- a/projects/business-intelligence/car-sales-workbook.xlsx
+++ b/projects/business-intelligence/car-sales-workbook.xlsx
@@ -4,9 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kama\Downloads\"/>
-    </mc:Choice>
+    <mc:Choice Requires="x15"/>
   </mc:AlternateContent>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7755"/>

</xml_diff>